<commit_message>
Add landlord variant + parameterized engine, mockup copy, catalog README
- Refactor build_tracker.py into a parameterized engine (VARIANTS dict); one
  source now builds both products and writes into per-product folders
- build_guide.py imports the same VARIANTS so guides can't drift from workbooks
- New product: Rental Property Tracker (long-term landlords) — xlsx, setup guide,
  listing copy, mockup copy. Verified totals: income 3575 / expenses 1395 / net 2180
- Add mockups.md (5-image copy) for both products
- Move engine scripts to products/ root; replace per-product README with a
  catalog-level products/README.md covering both products and the variant workflow
</commit_message>
<xml_diff>
--- a/products/str-tracker/Short-Term-Rental-Tracker.xlsx
+++ b/products/str-tracker/Short-Term-Rental-Tracker.xlsx
@@ -793,7 +793,7 @@
     <row r="14" ht="34" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>•  Duplicate the file per tax year (e.g. 'STR Tracker 2026').</t>
+          <t>•  Duplicate the file per tax year (e.g. 'Short-Term Rental 2026').</t>
         </is>
       </c>
     </row>
@@ -812,9 +812,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>